<commit_message>
Include sales channel in invoice line descriptions
Each PO line now reads 'Amazon Retail PO#XXXXX' or 'Ninja PO#XXXXXX'
(Ninja numbers keep their digits, folding the redundant PO prefix).
Also carries over the accountant's edits from their copy: 'Description'
/ 'Nasam Commission (SAR)' headers. All 133 lines and totals
re-verified (3710.35 SAR).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DFQiGGNTcyDsiA52SK6fSp
</commit_message>
<xml_diff>
--- a/po-invoices/commission_invoices.xlsx
+++ b/po-invoices/commission_invoices.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="172">
   <si>
     <t xml:space="preserve">Commission Invoices — Summary</t>
   </si>
@@ -154,19 +154,22 @@
     <t xml:space="preserve">Commission per PO = ROUND(Received × rate, 2).</t>
   </si>
   <si>
-    <t xml:space="preserve">PO Number</t>
+    <t xml:space="preserve">Description</t>
   </si>
   <si>
     <t xml:space="preserve">Commission %</t>
   </si>
   <si>
+    <t xml:space="preserve">Nasam Commission (SAR)</t>
+  </si>
+  <si>
     <t xml:space="preserve">INV-MARAH-2025-10  ·  Alaris Group  ·  Oct 2025</t>
   </si>
   <si>
-    <t xml:space="preserve">4TN3ZVSL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6PP725QB</t>
+    <t xml:space="preserve">Amazon Retail PO#4TN3ZVSL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6PP725QB</t>
   </si>
   <si>
     <t xml:space="preserve">Invoice total</t>
@@ -175,259 +178,259 @@
     <t xml:space="preserve">INV-MARAH-2025-11  ·  Alaris Group  ·  Nov 2025</t>
   </si>
   <si>
-    <t xml:space="preserve">2P93YCEF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6DY1IPME</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6WB73PWY</t>
+    <t xml:space="preserve">Amazon Retail PO#2P93YCEF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6DY1IPME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6WB73PWY</t>
   </si>
   <si>
     <t xml:space="preserve">INV-MARAH-2025-12  ·  Alaris Group  ·  Dec 2025</t>
   </si>
   <si>
-    <t xml:space="preserve">5EN36W7Q</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6CZVU75G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7M6TKRHR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6TDL7ZQP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6PSDP49U</t>
-  </si>
-  <si>
-    <t xml:space="preserve">797EACNS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6UBMEEFU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6V3M52MA</t>
+    <t xml:space="preserve">Amazon Retail PO#5EN36W7Q</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6CZVU75G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#7M6TKRHR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6TDL7ZQP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6PSDP49U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#797EACNS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6UBMEEFU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6V3M52MA</t>
   </si>
   <si>
     <t xml:space="preserve">INV-MARAH-2026-01  ·  Alaris Group  ·  Jan 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">6PH6KTZF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6S9RVIGN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8GLJBAPU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2B5T42JL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4MD92H1G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3NBXS26G</t>
+    <t xml:space="preserve">Amazon Retail PO#6PH6KTZF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6S9RVIGN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#8GLJBAPU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#2B5T42JL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#4MD92H1G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#3NBXS26G</t>
   </si>
   <si>
     <t xml:space="preserve">INV-MARAH-2026-02  ·  Alaris Group  ·  Feb 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">2776KBES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35A5IQ5O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2NMPDC6A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">63CNSAWW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2Q2CPLWE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">47SZZRUF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5CHSK8EF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8MME3VWE</t>
+    <t xml:space="preserve">Amazon Retail PO#2776KBES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#35A5IQ5O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#2NMPDC6A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#63CNSAWW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#2Q2CPLWE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#47SZZRUF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#5CHSK8EF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#8MME3VWE</t>
   </si>
   <si>
     <t xml:space="preserve">INV-MARAH-2026-03  ·  Alaris Group  ·  Mar 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">33272MDV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4VGJUUTB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">56ODNFEU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6BQUXPAB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7BB3BSGS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1KBAMBMY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12NKR58W</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6NWUZ15U</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7WF53VUB</t>
+    <t xml:space="preserve">Amazon Retail PO#33272MDV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#4VGJUUTB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#56ODNFEU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6BQUXPAB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#7BB3BSGS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#1KBAMBMY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#12NKR58W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6NWUZ15U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#7WF53VUB</t>
   </si>
   <si>
     <t xml:space="preserve">INV-MARAH-2026-04  ·  Alaris Group  ·  Apr 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">2I94WCYC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8GDABTDG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2FMA3P2X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5PE3P2GE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">45NJYTSJ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5A5RRTQI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2ZQ63SQZ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5C8HGLYP</t>
+    <t xml:space="preserve">Amazon Retail PO#2I94WCYC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#8GDABTDG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#2FMA3P2X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#5PE3P2GE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#45NJYTSJ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#5A5RRTQI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#2ZQ63SQZ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#5C8HGLYP</t>
   </si>
   <si>
     <t xml:space="preserve">INV-MARAH-2026-05  ·  Alaris Group  ·  May 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">4DM5ZX9S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5ZC4GIJB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6YXMCSBG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7FQQP3YA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4HJZN3HS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5YTDVHBW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">64ZRO2IW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4J9CPFNV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6G32T7VG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2B23XHGH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">57VZIBCA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">31WXVSCY</t>
+    <t xml:space="preserve">Amazon Retail PO#4DM5ZX9S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#5ZC4GIJB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6YXMCSBG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#7FQQP3YA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#4HJZN3HS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#5YTDVHBW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#64ZRO2IW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#4J9CPFNV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6G32T7VG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#2B23XHGH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#57VZIBCA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#31WXVSCY</t>
   </si>
   <si>
     <t xml:space="preserve">INV-MARAH-2026-06  ·  Alaris Group  ·  Jun 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">27HTOR4Q</t>
-  </si>
-  <si>
-    <t xml:space="preserve">77DN671B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6YXQJTKI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">78GBUJ1W</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8MHCMNQO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5R5X8LID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6DPTSK1M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2AMQJ9LR</t>
+    <t xml:space="preserve">Amazon Retail PO#27HTOR4Q</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#77DN671B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6YXQJTKI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#78GBUJ1W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#8MHCMNQO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#5R5X8LID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6DPTSK1M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#2AMQJ9LR</t>
   </si>
   <si>
     <t xml:space="preserve">INV-MARAH-2026-07  ·  Alaris Group  ·  Jul 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">6HIM13WU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7HEB8XWB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7X4T9L9X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">224Y4ETZ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3UR2NYQH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">74LAZ8YS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">65T5PXVI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6Z9UWMBO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7CS7ZUYR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5249UCBK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">64TUIPCQ</t>
+    <t xml:space="preserve">Amazon Retail PO#6HIM13WU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#7HEB8XWB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#7X4T9L9X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#224Y4ETZ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#3UR2NYQH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#74LAZ8YS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#65T5PXVI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6Z9UWMBO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#7CS7ZUYR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#5249UCBK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#64TUIPCQ</t>
   </si>
   <si>
     <t xml:space="preserve">INV-MARAH-2026-08  ·  Alaris Group  ·  Aug 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">13WKUXGQ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17WV7XMX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">53LUQGQJ</t>
+    <t xml:space="preserve">Amazon Retail PO#13WKUXGQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#17WV7XMX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#53LUQGQJ</t>
   </si>
   <si>
     <t xml:space="preserve">SONDOS — Commission Invoices — Customer: Alaris Group</t>
@@ -436,7 +439,7 @@
     <t xml:space="preserve">INV-SONDOS-2025-09  ·  Alaris Group  ·  Sep 2025</t>
   </si>
   <si>
-    <t xml:space="preserve">32EZOEJU</t>
+    <t xml:space="preserve">Amazon Retail PO#32EZOEJU</t>
   </si>
   <si>
     <t xml:space="preserve">INV-SONDOS-2025-10  ·  Alaris Group  ·  Oct 2025</t>
@@ -448,31 +451,31 @@
     <t xml:space="preserve">INV-SONDOS-2025-12  ·  Alaris Group  ·  Dec 2025</t>
   </si>
   <si>
-    <t xml:space="preserve">5ILLL7BX</t>
+    <t xml:space="preserve">Amazon Retail PO#5ILLL7BX</t>
   </si>
   <si>
     <t xml:space="preserve">INV-SONDOS-2026-01  ·  Alaris Group  ·  Jan 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">1G7W4QOA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4Q9D66FC</t>
+    <t xml:space="preserve">Amazon Retail PO#1G7W4QOA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#4Q9D66FC</t>
   </si>
   <si>
     <t xml:space="preserve">INV-SONDOS-2026-02  ·  Alaris Group  ·  Feb 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">85YJNW7Z</t>
+    <t xml:space="preserve">Amazon Retail PO#85YJNW7Z</t>
   </si>
   <si>
     <t xml:space="preserve">INV-SONDOS-2026-03  ·  Alaris Group  ·  Mar 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">3EO1QUXF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1Y1T5K2Z</t>
+    <t xml:space="preserve">Amazon Retail PO#3EO1QUXF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#1Y1T5K2Z</t>
   </si>
   <si>
     <t xml:space="preserve">INV-SONDOS-2026-04  ·  Alaris Group  ·  Apr 2026</t>
@@ -484,19 +487,19 @@
     <t xml:space="preserve">INV-SONDOS-2026-06  ·  Alaris Group  ·  Jun 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">34RW3MWX</t>
+    <t xml:space="preserve">Amazon Retail PO#34RW3MWX</t>
   </si>
   <si>
     <t xml:space="preserve">INV-SONDOS-2026-07  ·  Alaris Group  ·  Jul 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">2VS58KHE</t>
+    <t xml:space="preserve">Amazon Retail PO#2VS58KHE</t>
   </si>
   <si>
     <t xml:space="preserve">INV-SONDOS-2026-08  ·  Alaris Group  ·  Aug 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">1F6WGJRN</t>
+    <t xml:space="preserve">Amazon Retail PO#1F6WGJRN</t>
   </si>
   <si>
     <t xml:space="preserve">Wadi Halfa — Commission Invoices — Customer: Wadi Halfa</t>
@@ -505,37 +508,37 @@
     <t xml:space="preserve">INV-WADIHALFA-2026-06  ·  Wadi Halfa  ·  Jun 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">523FHETX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4KDCOEYS</t>
+    <t xml:space="preserve">Amazon Retail PO#523FHETX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#4KDCOEYS</t>
   </si>
   <si>
     <t xml:space="preserve">INV-WADIHALFA-2026-07  ·  Wadi Halfa  ·  Jul 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">PO2600607394</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PO2600607555</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6WAWK77S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PO2600629370</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PO2600629540</t>
+    <t xml:space="preserve">Ninja PO#2600607394</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ninja PO#2600607555</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Retail PO#6WAWK77S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ninja PO#2600629370</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ninja PO#2600629540</t>
   </si>
   <si>
     <t xml:space="preserve">INV-WADIHALFA-2026-08  ·  Wadi Halfa  ·  Aug 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">PO2600651634</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PO2600651819</t>
+    <t xml:space="preserve">Ninja PO#2600651634</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ninja PO#2600651819</t>
   </si>
 </sst>
 </file>
@@ -1782,11 +1785,11 @@
   <dimension ref="A1:E114"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1819,12 +1822,12 @@
         <v>44</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>8</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B5" s="13"/>
       <c r="C5" s="13"/>
@@ -1833,7 +1836,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B6" s="6" t="n">
         <v>45931</v>
@@ -1852,7 +1855,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B7" s="6" t="n">
         <v>45931</v>
@@ -1871,7 +1874,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="10" t="n">
@@ -1886,7 +1889,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
@@ -1895,7 +1898,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B11" s="6" t="n">
         <v>45962</v>
@@ -1914,7 +1917,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B12" s="6" t="n">
         <v>45962</v>
@@ -1933,7 +1936,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B13" s="6" t="n">
         <v>45962</v>
@@ -1952,7 +1955,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="10" t="n">
@@ -1967,7 +1970,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
@@ -1976,7 +1979,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B17" s="6" t="n">
         <v>45992</v>
@@ -1995,7 +1998,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B18" s="6" t="n">
         <v>45992</v>
@@ -2014,7 +2017,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B19" s="6" t="n">
         <v>45992</v>
@@ -2033,7 +2036,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B20" s="6" t="n">
         <v>45992</v>
@@ -2052,7 +2055,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B21" s="6" t="n">
         <v>45992</v>
@@ -2071,7 +2074,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B22" s="6" t="n">
         <v>45992</v>
@@ -2090,7 +2093,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B23" s="6" t="n">
         <v>45992</v>
@@ -2109,7 +2112,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B24" s="6" t="n">
         <v>45992</v>
@@ -2128,7 +2131,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="10" t="n">
@@ -2143,7 +2146,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
@@ -2152,7 +2155,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B28" s="6" t="n">
         <v>46023</v>
@@ -2171,7 +2174,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B29" s="6" t="n">
         <v>46023</v>
@@ -2190,7 +2193,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B30" s="6" t="n">
         <v>46023</v>
@@ -2209,7 +2212,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B31" s="6" t="n">
         <v>46023</v>
@@ -2228,7 +2231,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B32" s="6" t="n">
         <v>46023</v>
@@ -2247,7 +2250,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B33" s="6" t="n">
         <v>46023</v>
@@ -2266,7 +2269,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B34" s="8"/>
       <c r="C34" s="10" t="n">
@@ -2281,7 +2284,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B36" s="13"/>
       <c r="C36" s="13"/>
@@ -2290,7 +2293,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B37" s="6" t="n">
         <v>46054</v>
@@ -2309,7 +2312,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B38" s="6" t="n">
         <v>46054</v>
@@ -2328,7 +2331,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B39" s="6" t="n">
         <v>46054</v>
@@ -2347,7 +2350,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B40" s="6" t="n">
         <v>46054</v>
@@ -2366,7 +2369,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B41" s="6" t="n">
         <v>46054</v>
@@ -2385,7 +2388,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B42" s="6" t="n">
         <v>46054</v>
@@ -2404,7 +2407,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B43" s="6" t="n">
         <v>46054</v>
@@ -2423,7 +2426,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B44" s="6" t="n">
         <v>46054</v>
@@ -2442,7 +2445,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B45" s="8"/>
       <c r="C45" s="10" t="n">
@@ -2457,7 +2460,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B47" s="13"/>
       <c r="C47" s="13"/>
@@ -2466,7 +2469,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B48" s="6" t="n">
         <v>46082</v>
@@ -2485,7 +2488,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B49" s="6" t="n">
         <v>46082</v>
@@ -2504,7 +2507,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B50" s="6" t="n">
         <v>46082</v>
@@ -2523,7 +2526,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B51" s="6" t="n">
         <v>46082</v>
@@ -2542,7 +2545,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B52" s="6" t="n">
         <v>46082</v>
@@ -2561,7 +2564,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B53" s="6" t="n">
         <v>46082</v>
@@ -2580,7 +2583,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B54" s="6" t="n">
         <v>46082</v>
@@ -2599,7 +2602,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B55" s="6" t="n">
         <v>46082</v>
@@ -2618,7 +2621,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B56" s="6" t="n">
         <v>46082</v>
@@ -2637,7 +2640,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B57" s="8"/>
       <c r="C57" s="10" t="n">
@@ -2652,7 +2655,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B59" s="13"/>
       <c r="C59" s="13"/>
@@ -2661,7 +2664,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B60" s="6" t="n">
         <v>46113</v>
@@ -2680,7 +2683,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B61" s="6" t="n">
         <v>46113</v>
@@ -2699,7 +2702,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B62" s="6" t="n">
         <v>46113</v>
@@ -2718,7 +2721,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B63" s="6" t="n">
         <v>46113</v>
@@ -2737,7 +2740,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B64" s="6" t="n">
         <v>46113</v>
@@ -2756,7 +2759,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B65" s="6" t="n">
         <v>46113</v>
@@ -2775,7 +2778,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B66" s="6" t="n">
         <v>46113</v>
@@ -2794,7 +2797,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B67" s="6" t="n">
         <v>46113</v>
@@ -2813,7 +2816,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B68" s="8"/>
       <c r="C68" s="10" t="n">
@@ -2828,7 +2831,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B70" s="13"/>
       <c r="C70" s="13"/>
@@ -2837,7 +2840,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B71" s="6" t="n">
         <v>46143</v>
@@ -2856,7 +2859,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B72" s="6" t="n">
         <v>46143</v>
@@ -2875,7 +2878,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B73" s="6" t="n">
         <v>46143</v>
@@ -2894,7 +2897,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B74" s="6" t="n">
         <v>46143</v>
@@ -2913,7 +2916,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B75" s="6" t="n">
         <v>46143</v>
@@ -2932,7 +2935,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B76" s="6" t="n">
         <v>46143</v>
@@ -2951,7 +2954,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B77" s="6" t="n">
         <v>46143</v>
@@ -2970,7 +2973,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B78" s="6" t="n">
         <v>46143</v>
@@ -2989,7 +2992,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B79" s="6" t="n">
         <v>46143</v>
@@ -3008,7 +3011,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B80" s="6" t="n">
         <v>46143</v>
@@ -3027,7 +3030,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B81" s="6" t="n">
         <v>46143</v>
@@ -3046,7 +3049,7 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B82" s="6" t="n">
         <v>46143</v>
@@ -3065,7 +3068,7 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B83" s="8"/>
       <c r="C83" s="10" t="n">
@@ -3080,7 +3083,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B85" s="13"/>
       <c r="C85" s="13"/>
@@ -3089,7 +3092,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B86" s="6" t="n">
         <v>46174</v>
@@ -3108,7 +3111,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B87" s="6" t="n">
         <v>46174</v>
@@ -3127,7 +3130,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B88" s="6" t="n">
         <v>46174</v>
@@ -3146,7 +3149,7 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B89" s="6" t="n">
         <v>46174</v>
@@ -3165,7 +3168,7 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B90" s="6" t="n">
         <v>46174</v>
@@ -3184,7 +3187,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B91" s="6" t="n">
         <v>46174</v>
@@ -3203,7 +3206,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B92" s="6" t="n">
         <v>46174</v>
@@ -3222,7 +3225,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B93" s="6" t="n">
         <v>46174</v>
@@ -3241,7 +3244,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B94" s="8"/>
       <c r="C94" s="10" t="n">
@@ -3256,7 +3259,7 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B96" s="13"/>
       <c r="C96" s="13"/>
@@ -3265,7 +3268,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B97" s="6" t="n">
         <v>46204</v>
@@ -3284,7 +3287,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B98" s="6" t="n">
         <v>46204</v>
@@ -3303,7 +3306,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B99" s="6" t="n">
         <v>46204</v>
@@ -3322,7 +3325,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B100" s="6" t="n">
         <v>46204</v>
@@ -3341,7 +3344,7 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B101" s="6" t="n">
         <v>46204</v>
@@ -3360,7 +3363,7 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B102" s="6" t="n">
         <v>46204</v>
@@ -3379,7 +3382,7 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B103" s="6" t="n">
         <v>46204</v>
@@ -3398,7 +3401,7 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B104" s="6" t="n">
         <v>46204</v>
@@ -3417,7 +3420,7 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B105" s="6" t="n">
         <v>46204</v>
@@ -3436,7 +3439,7 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B106" s="6" t="n">
         <v>46204</v>
@@ -3455,7 +3458,7 @@
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B107" s="6" t="n">
         <v>46204</v>
@@ -3474,7 +3477,7 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B108" s="8"/>
       <c r="C108" s="10" t="n">
@@ -3489,7 +3492,7 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B110" s="13"/>
       <c r="C110" s="13"/>
@@ -3498,7 +3501,7 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B111" s="6" t="n">
         <v>46235</v>
@@ -3517,7 +3520,7 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B112" s="6" t="n">
         <v>46235</v>
@@ -3536,7 +3539,7 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B113" s="6" t="n">
         <v>46235</v>
@@ -3555,7 +3558,7 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B114" s="8"/>
       <c r="C114" s="10" t="n">
@@ -3587,16 +3590,16 @@
   <dimension ref="A1:E85"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3624,12 +3627,12 @@
         <v>44</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>8</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B5" s="13"/>
       <c r="C5" s="13"/>
@@ -3638,7 +3641,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B6" s="6" t="n">
         <v>45901</v>
@@ -3657,7 +3660,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="10" t="n">
@@ -3672,7 +3675,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B9" s="13"/>
       <c r="C9" s="13"/>
@@ -3681,7 +3684,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B10" s="6" t="n">
         <v>45931</v>
@@ -3700,7 +3703,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="10" t="n">
@@ -3715,7 +3718,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
@@ -3724,7 +3727,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B14" s="6" t="n">
         <v>45962</v>
@@ -3743,7 +3746,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B15" s="6" t="n">
         <v>45962</v>
@@ -3762,7 +3765,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="10" t="n">
@@ -3777,7 +3780,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
@@ -3786,7 +3789,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B19" s="6" t="n">
         <v>45992</v>
@@ -3805,7 +3808,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B20" s="6" t="n">
         <v>45992</v>
@@ -3824,7 +3827,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B21" s="6" t="n">
         <v>45992</v>
@@ -3843,7 +3846,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B22" s="6" t="n">
         <v>45992</v>
@@ -3862,7 +3865,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B23" s="6" t="n">
         <v>45992</v>
@@ -3881,7 +3884,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="10" t="n">
@@ -3896,7 +3899,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
@@ -3905,7 +3908,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B27" s="6" t="n">
         <v>46023</v>
@@ -3924,7 +3927,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B28" s="6" t="n">
         <v>46023</v>
@@ -3943,7 +3946,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B29" s="6" t="n">
         <v>46023</v>
@@ -3962,7 +3965,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B30" s="6" t="n">
         <v>46023</v>
@@ -3981,7 +3984,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B31" s="8"/>
       <c r="C31" s="10" t="n">
@@ -3996,7 +3999,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B33" s="13"/>
       <c r="C33" s="13"/>
@@ -4005,7 +4008,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B34" s="6" t="n">
         <v>46054</v>
@@ -4024,7 +4027,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B35" s="6" t="n">
         <v>46054</v>
@@ -4043,7 +4046,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B36" s="6" t="n">
         <v>46054</v>
@@ -4062,7 +4065,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B37" s="6" t="n">
         <v>46054</v>
@@ -4081,7 +4084,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B38" s="6" t="n">
         <v>46054</v>
@@ -4100,7 +4103,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B39" s="8"/>
       <c r="C39" s="10" t="n">
@@ -4115,7 +4118,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="13" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B41" s="13"/>
       <c r="C41" s="13"/>
@@ -4124,7 +4127,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B42" s="6" t="n">
         <v>46082</v>
@@ -4143,7 +4146,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B43" s="6" t="n">
         <v>46082</v>
@@ -4162,7 +4165,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B44" s="6" t="n">
         <v>46082</v>
@@ -4181,7 +4184,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B45" s="6" t="n">
         <v>46082</v>
@@ -4200,7 +4203,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B46" s="6" t="n">
         <v>46082</v>
@@ -4219,7 +4222,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B47" s="6" t="n">
         <v>46082</v>
@@ -4238,7 +4241,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B48" s="6" t="n">
         <v>46082</v>
@@ -4257,7 +4260,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="10" t="n">
@@ -4272,7 +4275,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B51" s="13"/>
       <c r="C51" s="13"/>
@@ -4281,7 +4284,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B52" s="6" t="n">
         <v>46113</v>
@@ -4300,7 +4303,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B53" s="6" t="n">
         <v>46113</v>
@@ -4319,7 +4322,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B54" s="6" t="n">
         <v>46113</v>
@@ -4338,7 +4341,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B55" s="6" t="n">
         <v>46113</v>
@@ -4357,7 +4360,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="10" t="n">
@@ -4372,7 +4375,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B58" s="13"/>
       <c r="C58" s="13"/>
@@ -4381,7 +4384,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B59" s="6" t="n">
         <v>46143</v>
@@ -4400,7 +4403,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B60" s="6" t="n">
         <v>46143</v>
@@ -4419,7 +4422,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B61" s="6" t="n">
         <v>46143</v>
@@ -4438,7 +4441,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B62" s="6" t="n">
         <v>46143</v>
@@ -4457,7 +4460,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B63" s="6" t="n">
         <v>46143</v>
@@ -4476,7 +4479,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="10" t="n">
@@ -4491,7 +4494,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="13" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B66" s="13"/>
       <c r="C66" s="13"/>
@@ -4500,7 +4503,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B67" s="6" t="n">
         <v>46174</v>
@@ -4519,7 +4522,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B68" s="6" t="n">
         <v>46174</v>
@@ -4538,7 +4541,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B69" s="6" t="n">
         <v>46174</v>
@@ -4557,7 +4560,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B70" s="6" t="n">
         <v>46174</v>
@@ -4576,7 +4579,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B71" s="6" t="n">
         <v>46174</v>
@@ -4595,7 +4598,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B72" s="6" t="n">
         <v>46174</v>
@@ -4614,7 +4617,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B73" s="8"/>
       <c r="C73" s="10" t="n">
@@ -4629,7 +4632,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="13" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B75" s="13"/>
       <c r="C75" s="13"/>
@@ -4638,7 +4641,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B76" s="6" t="n">
         <v>46204</v>
@@ -4657,7 +4660,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B77" s="6" t="n">
         <v>46204</v>
@@ -4676,7 +4679,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B78" s="6" t="n">
         <v>46204</v>
@@ -4695,7 +4698,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B79" s="6" t="n">
         <v>46204</v>
@@ -4714,7 +4717,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B80" s="6" t="n">
         <v>46204</v>
@@ -4733,7 +4736,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B81" s="8"/>
       <c r="C81" s="10" t="n">
@@ -4748,7 +4751,7 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="13" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B83" s="13"/>
       <c r="C83" s="13"/>
@@ -4757,7 +4760,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B84" s="6" t="n">
         <v>46235</v>
@@ -4776,7 +4779,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B85" s="8"/>
       <c r="C85" s="10" t="n">
@@ -4808,16 +4811,16 @@
   <dimension ref="A1:E21"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4845,12 +4848,12 @@
         <v>44</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>8</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B5" s="13"/>
       <c r="C5" s="13"/>
@@ -4859,7 +4862,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B6" s="6" t="n">
         <v>46174</v>
@@ -4878,7 +4881,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B7" s="6" t="n">
         <v>46174</v>
@@ -4897,7 +4900,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="10" t="n">
@@ -4912,7 +4915,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
@@ -4921,7 +4924,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B11" s="6" t="n">
         <v>46204</v>
@@ -4940,7 +4943,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B12" s="6" t="n">
         <v>46204</v>
@@ -4959,7 +4962,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B13" s="6" t="n">
         <v>46204</v>
@@ -4978,7 +4981,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B14" s="6" t="n">
         <v>46204</v>
@@ -4997,7 +5000,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B15" s="6" t="n">
         <v>46204</v>
@@ -5016,7 +5019,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="10" t="n">
@@ -5031,7 +5034,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
@@ -5040,7 +5043,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B19" s="6" t="n">
         <v>46235</v>
@@ -5059,7 +5062,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B20" s="6" t="n">
         <v>46235</v>
@@ -5078,7 +5081,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="10" t="n">

</xml_diff>